<commit_message>
setting up for packaging using pyinstaller
</commit_message>
<xml_diff>
--- a/data/Scholarship_Assessor_Data.xlsx
+++ b/data/Scholarship_Assessor_Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f3ac2bf50d090347/Documents/Python/Neontribe/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f3ac2bf50d090347/Documents/Python/Neontribe/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{0010BE3C-1B6C-440B-A49F-88E907AB69C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0ED7D407-0796-4950-88A5-44124CBC4016}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{0010BE3C-1B6C-440B-A49F-88E907AB69C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B303518C-915E-4459-A5FE-78404DCAFCA2}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{618B0539-A1B0-495B-B98C-8ABAAC5394CB}"/>
+    <workbookView minimized="1" xWindow="1800" yWindow="1120" windowWidth="9640" windowHeight="8960" xr2:uid="{618B0539-A1B0-495B-B98C-8ABAAC5394CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Scholarship_Assessor_Data" sheetId="1" r:id="rId1"/>
@@ -1392,10 +1392,10 @@
         <v>0</v>
       </c>
       <c r="B1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D1">
         <v>3</v>
@@ -1416,7 +1416,7 @@
         <v>8</v>
       </c>
       <c r="J1">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K1">
         <v>10</v>
@@ -1547,10 +1547,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D2" t="s">
         <v>14</v>
@@ -1571,7 +1571,7 @@
         <v>34</v>
       </c>
       <c r="J2" t="s">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="K2" t="s">
         <v>44</v>
@@ -1702,10 +1702,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s">
         <v>15</v>
@@ -1726,7 +1726,7 @@
         <v>35</v>
       </c>
       <c r="J3" t="s">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="K3" t="s">
         <v>45</v>
@@ -1857,10 +1857,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="D4" t="s">
         <v>16</v>
@@ -1881,7 +1881,7 @@
         <v>36</v>
       </c>
       <c r="J4" t="s">
-        <v>42</v>
+        <v>7</v>
       </c>
       <c r="K4" t="s">
         <v>12</v>
@@ -2012,10 +2012,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
         <v>17</v>
@@ -2036,7 +2036,7 @@
         <v>37</v>
       </c>
       <c r="J5" t="s">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="K5" t="s">
         <v>22</v>
@@ -2170,7 +2170,7 @@
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
         <v>18</v>
@@ -2191,7 +2191,7 @@
         <v>38</v>
       </c>
       <c r="J6" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="K6" t="s">
         <v>9</v>
@@ -2325,7 +2325,7 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="D7" t="s">
         <v>9</v>
@@ -2346,7 +2346,7 @@
         <v>39</v>
       </c>
       <c r="J7" t="s">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="K7" t="s">
         <v>9</v>
@@ -2474,5 +2474,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>